<commit_message>
Phase 0: retain Schedule Import conflict warning
</commit_message>
<xml_diff>
--- a/docs/qt-rewrite/visual-baseline/release/large-schedule-import-boundary/generated-large-schedule-import.xlsx
+++ b/docs/qt-rewrite/visual-baseline/release/large-schedule-import-boundary/generated-large-schedule-import.xlsx
@@ -200,10 +200,10 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+          <t>3:00~3:55</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>김선생 (301)
 E5-Artemis</t>
@@ -213,10 +213,10 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>5:00~5:55</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
+          <t>3:00~3:55</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>김선생 (301)
 E6-Helios</t>
@@ -226,10 +226,10 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+          <t>3:00~3:55</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>김선생 (301)
 M1-Elephantus</t>
@@ -239,10 +239,10 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>7:00~7:55</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
+          <t>4:00~4:55</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>이선생 (302)
 E4-Theseus</t>
@@ -252,10 +252,10 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>8:00~8:55</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+          <t>4:00~4:55</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
         <is>
           <t>이선생 (302)
 E5-Artemis</t>
@@ -265,7 +265,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
+          <t>4:00~4:55</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -281,7 +281,7 @@
           <t>4:00~4:55</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>이선생 (302)
 M1-Elephantus</t>
@@ -294,7 +294,7 @@
           <t>5:00~5:55</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>박선생 (303)
 E4-Theseus</t>
@@ -304,10 +304,10 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
+          <t>5:00~5:55</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t>박선생 (303)
 E5-Artemis</t>
@@ -317,10 +317,10 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>7:00~7:55</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+          <t>5:00~5:55</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
         <is>
           <t>박선생 (303)
 E6-Helios</t>
@@ -330,10 +330,10 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8:00~8:55</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
+          <t>5:00~5:55</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>박선생 (303)
 M1-Elephantus</t>
@@ -343,10 +343,10 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
+          <t>6:00~6:55</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>최선생 (304)
 E4-Theseus</t>
@@ -356,7 +356,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
+          <t>6:00~6:55</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -369,10 +369,10 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>5:00~5:55</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
+          <t>6:00~6:55</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>최선생 (304)
 E6-Helios</t>
@@ -385,7 +385,7 @@
           <t>6:00~6:55</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>최선생 (304)
 M1-Elephantus</t>
@@ -398,7 +398,7 @@
           <t>7:00~7:55</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>정선생 (305)
 E4-Theseus</t>
@@ -408,10 +408,10 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>8:00~8:55</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
+          <t>7:00~7:55</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
         <is>
           <t>정선생 (305)
 E5-Artemis</t>
@@ -421,10 +421,10 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
+          <t>7:00~7:55</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
         <is>
           <t>정선생 (305)
 E6-Helios</t>
@@ -434,7 +434,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
+          <t>7:00~7:55</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -447,7 +447,7 @@
     <row r="2">
       <c r="H2" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
+          <t>8:00~8:55</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -460,10 +460,10 @@
     <row r="3">
       <c r="H3" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
+          <t>8:00~8:55</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>한선생 (306)
 E5-Artemis</t>
@@ -473,10 +473,10 @@
     <row r="4">
       <c r="H4" t="inlineStr">
         <is>
-          <t>5:00~5:55</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
+          <t>8:00~8:55</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>한선생 (306)
 E6-Helios</t>
@@ -486,10 +486,10 @@
     <row r="5">
       <c r="H5" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
+          <t>8:00~8:55</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>한선생 (306)
 M1-Elephantus</t>
@@ -499,10 +499,10 @@
     <row r="6">
       <c r="H6" t="inlineStr">
         <is>
-          <t>7:00~7:55</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
+          <t>3:00~3:55</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>강선생 (307)
 E4-Theseus</t>
@@ -512,10 +512,10 @@
     <row r="7">
       <c r="H7" t="inlineStr">
         <is>
-          <t>8:00~8:55</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
+          <t>3:00~3:55</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>강선생 (307)
 E5-Artemis</t>
@@ -538,10 +538,10 @@
     <row r="9">
       <c r="H9" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
+          <t>3:00~3:55</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>강선생 (307)
 M1-Elephantus</t>
@@ -551,10 +551,10 @@
     <row r="10">
       <c r="H10" t="inlineStr">
         <is>
-          <t>5:00~5:55</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
+          <t>4:00~4:55</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>윤선생 (308)
 E4-Theseus</t>
@@ -564,10 +564,10 @@
     <row r="11">
       <c r="H11" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
+          <t>4:00~4:55</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>윤선생 (308)
 E5-Artemis</t>
@@ -577,10 +577,10 @@
     <row r="12">
       <c r="H12" t="inlineStr">
         <is>
-          <t>7:00~7:55</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
+          <t>4:00~4:55</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
         <is>
           <t>윤선생 (308)
 E6-Helios</t>
@@ -590,10 +590,10 @@
     <row r="13">
       <c r="H13" t="inlineStr">
         <is>
-          <t>8:00~8:55</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
+          <t>4:00~4:55</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t>윤선생 (308)
 M1-Elephantus</t>
@@ -603,10 +603,10 @@
     <row r="14">
       <c r="H14" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
+          <t>5:00~5:55</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>조선생 (309)
 E4-Theseus</t>
@@ -616,7 +616,7 @@
     <row r="15">
       <c r="H15" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
+          <t>5:00~5:55</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -632,7 +632,7 @@
           <t>5:00~5:55</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>조선생 (309)
 E6-Helios</t>
@@ -642,10 +642,10 @@
     <row r="17">
       <c r="H17" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
+          <t>5:00~5:55</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>조선생 (309)
 M1-Elephantus</t>
@@ -655,10 +655,10 @@
     <row r="18">
       <c r="H18" t="inlineStr">
         <is>
-          <t>7:00~7:55</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
+          <t>6:00~6:55</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>임선생 (310)
 E4-Theseus</t>
@@ -668,10 +668,10 @@
     <row r="19">
       <c r="H19" t="inlineStr">
         <is>
-          <t>8:00~8:55</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
+          <t>6:00~6:55</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
         <is>
           <t>임선생 (310)
 E5-Artemis</t>
@@ -681,10 +681,10 @@
     <row r="20">
       <c r="H20" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
+          <t>6:00~6:55</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
         <is>
           <t>임선생 (310)
 E6-Helios</t>
@@ -694,7 +694,7 @@
     <row r="21">
       <c r="H21" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
+          <t>6:00~6:55</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="2">
       <c r="O2" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
+          <t>7:00~7:55</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -720,10 +720,10 @@
     <row r="3">
       <c r="O3" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
+          <t>7:00~7:55</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
         <is>
           <t>장선생 (311)
 E5-Artemis</t>
@@ -733,10 +733,10 @@
     <row r="4">
       <c r="O4" t="inlineStr">
         <is>
-          <t>5:00~5:55</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
+          <t>7:00~7:55</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
         <is>
           <t>장선생 (311)
 E6-Helios</t>
@@ -746,10 +746,10 @@
     <row r="5">
       <c r="O5" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
+          <t>7:00~7:55</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
         <is>
           <t>장선생 (311)
 M1-Elephantus</t>
@@ -759,10 +759,10 @@
     <row r="6">
       <c r="O6" t="inlineStr">
         <is>
-          <t>7:00~7:55</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
+          <t>8:00~8:55</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>오선생 (312)
 E4-Theseus</t>
@@ -775,7 +775,7 @@
           <t>8:00~8:55</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>오선생 (312)
 E5-Artemis</t>
@@ -785,7 +785,7 @@
     <row r="8">
       <c r="O8" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
+          <t>8:00~8:55</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -798,10 +798,10 @@
     <row r="9">
       <c r="O9" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
+          <t>8:00~8:55</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>오선생 (312)
 M1-Elephantus</t>
@@ -811,10 +811,10 @@
     <row r="10">
       <c r="O10" t="inlineStr">
         <is>
-          <t>5:00~5:55</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
+          <t>3:00~3:55</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
         <is>
           <t>서선생 (313)
 E4-Theseus</t>
@@ -824,10 +824,10 @@
     <row r="11">
       <c r="O11" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
+          <t>3:00~3:55</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
         <is>
           <t>서선생 (313)
 E5-Artemis</t>
@@ -837,10 +837,10 @@
     <row r="12">
       <c r="O12" t="inlineStr">
         <is>
-          <t>7:00~7:55</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
+          <t>3:00~3:55</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
         <is>
           <t>서선생 (313)
 E6-Helios</t>
@@ -850,10 +850,10 @@
     <row r="13">
       <c r="O13" t="inlineStr">
         <is>
-          <t>8:00~8:55</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
+          <t>3:00~3:55</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
         <is>
           <t>서선생 (313)
 M1-Elephantus</t>
@@ -863,10 +863,10 @@
     <row r="14">
       <c r="O14" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
+          <t>4:00~4:55</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
         <is>
           <t>신선생 (314)
 E4-Theseus</t>
@@ -889,10 +889,10 @@
     <row r="16">
       <c r="O16" t="inlineStr">
         <is>
-          <t>5:00~5:55</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
+          <t>4:00~4:55</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
         <is>
           <t>신선생 (314)
 E6-Helios</t>
@@ -902,10 +902,10 @@
     <row r="17">
       <c r="O17" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
+          <t>4:00~4:55</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
         <is>
           <t>신선생 (314)
 M1-Elephantus</t>
@@ -915,10 +915,10 @@
     <row r="18">
       <c r="O18" t="inlineStr">
         <is>
-          <t>7:00~7:55</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
+          <t>5:00~5:55</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
         <is>
           <t>권선생 (315)
 E4-Theseus</t>
@@ -928,10 +928,10 @@
     <row r="19">
       <c r="O19" t="inlineStr">
         <is>
-          <t>8:00~8:55</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
+          <t>5:00~5:55</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
         <is>
           <t>권선생 (315)
 E5-Artemis</t>
@@ -941,10 +941,10 @@
     <row r="20">
       <c r="O20" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
+          <t>5:00~5:55</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
         <is>
           <t>권선생 (315)
 E6-Helios</t>
@@ -954,7 +954,7 @@
     <row r="21">
       <c r="O21" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
+          <t>5:00~5:55</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -967,7 +967,7 @@
     <row r="2">
       <c r="V2" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
+          <t>6:00~6:55</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -980,10 +980,10 @@
     <row r="3">
       <c r="V3" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
+          <t>6:00~6:55</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
         <is>
           <t>황선생 (316)
 E5-Artemis</t>
@@ -993,10 +993,10 @@
     <row r="4">
       <c r="V4" t="inlineStr">
         <is>
-          <t>5:00~5:55</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
+          <t>6:00~6:55</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
         <is>
           <t>황선생 (316)
 E6-Helios</t>
@@ -1009,7 +1009,7 @@
           <t>6:00~6:55</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>황선생 (316)
 M1-Elephantus</t>
@@ -1022,7 +1022,7 @@
           <t>7:00~7:55</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>안선생 (317)
 E4-Theseus</t>
@@ -1032,10 +1032,10 @@
     <row r="7">
       <c r="V7" t="inlineStr">
         <is>
-          <t>8:00~8:55</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
+          <t>7:00~7:55</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
         <is>
           <t>안선생 (317)
 E5-Artemis</t>
@@ -1045,7 +1045,7 @@
     <row r="8">
       <c r="V8" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
+          <t>7:00~7:55</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -1058,10 +1058,10 @@
     <row r="9">
       <c r="V9" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
-        </is>
-      </c>
-      <c r="Y9" t="inlineStr">
+          <t>7:00~7:55</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
         <is>
           <t>안선생 (317)
 M1-Elephantus</t>
@@ -1071,10 +1071,10 @@
     <row r="10">
       <c r="V10" t="inlineStr">
         <is>
-          <t>5:00~5:55</t>
-        </is>
-      </c>
-      <c r="Z10" t="inlineStr">
+          <t>8:00~8:55</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
         <is>
           <t>송선생 (318)
 E4-Theseus</t>
@@ -1084,10 +1084,10 @@
     <row r="11">
       <c r="V11" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="AA11" t="inlineStr">
+          <t>8:00~8:55</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
         <is>
           <t>송선생 (318)
 E5-Artemis</t>
@@ -1097,10 +1097,10 @@
     <row r="12">
       <c r="V12" t="inlineStr">
         <is>
-          <t>7:00~7:55</t>
-        </is>
-      </c>
-      <c r="W12" t="inlineStr">
+          <t>8:00~8:55</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
         <is>
           <t>송선생 (318)
 E6-Helios</t>
@@ -1113,7 +1113,7 @@
           <t>8:00~8:55</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="Y13" t="inlineStr">
         <is>
           <t>송선생 (318)
 M1-Elephantus</t>
@@ -1126,7 +1126,7 @@
           <t>3:00~3:55</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr">
+      <c r="Z14" t="inlineStr">
         <is>
           <t>류선생 (319)
 E4-Theseus</t>
@@ -1136,7 +1136,7 @@
     <row r="15">
       <c r="V15" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
+          <t>3:00~3:55</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
@@ -1149,10 +1149,10 @@
     <row r="16">
       <c r="V16" t="inlineStr">
         <is>
-          <t>5:00~5:55</t>
-        </is>
-      </c>
-      <c r="AA16" t="inlineStr">
+          <t>3:00~3:55</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
         <is>
           <t>류선생 (319)
 E6-Helios</t>
@@ -1162,10 +1162,10 @@
     <row r="17">
       <c r="V17" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr">
+          <t>3:00~3:55</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
         <is>
           <t>류선생 (319)
 M1-Elephantus</t>
@@ -1175,10 +1175,10 @@
     <row r="18">
       <c r="V18" t="inlineStr">
         <is>
-          <t>7:00~7:55</t>
-        </is>
-      </c>
-      <c r="X18" t="inlineStr">
+          <t>4:00~4:55</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
         <is>
           <t>전선생 (320)
 E4-Theseus</t>
@@ -1188,10 +1188,10 @@
     <row r="19">
       <c r="V19" t="inlineStr">
         <is>
-          <t>8:00~8:55</t>
-        </is>
-      </c>
-      <c r="Y19" t="inlineStr">
+          <t>4:00~4:55</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
         <is>
           <t>전선생 (320)
 E5-Artemis</t>
@@ -1201,10 +1201,10 @@
     <row r="20">
       <c r="V20" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
-        </is>
-      </c>
-      <c r="Z20" t="inlineStr">
+          <t>4:00~4:55</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
         <is>
           <t>전선생 (320)
 E6-Helios</t>
@@ -1227,7 +1227,7 @@
     <row r="2">
       <c r="AC2" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
+          <t>5:00~5:55</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -1240,10 +1240,10 @@
     <row r="3">
       <c r="AC3" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
+          <t>5:00~5:55</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
         <is>
           <t>홍선생 (321)
 E5-Artemis</t>
@@ -1256,7 +1256,7 @@
           <t>5:00~5:55</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>홍선생 (321)
 E6-Helios</t>
@@ -1266,10 +1266,10 @@
     <row r="5">
       <c r="AC5" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
+          <t>5:00~5:55</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
         <is>
           <t>홍선생 (321)
 M1-Elephantus</t>
@@ -1279,10 +1279,10 @@
     <row r="6">
       <c r="AC6" t="inlineStr">
         <is>
-          <t>7:00~7:55</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
+          <t>6:00~6:55</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
         <is>
           <t>문선생 (322)
 E4-Theseus</t>
@@ -1292,10 +1292,10 @@
     <row r="7">
       <c r="AC7" t="inlineStr">
         <is>
-          <t>8:00~8:55</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
+          <t>6:00~6:55</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
         <is>
           <t>문선생 (322)
 E5-Artemis</t>
@@ -1305,7 +1305,7 @@
     <row r="8">
       <c r="AC8" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
+          <t>6:00~6:55</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
@@ -1318,10 +1318,10 @@
     <row r="9">
       <c r="AC9" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
-        </is>
-      </c>
-      <c r="AF9" t="inlineStr">
+          <t>6:00~6:55</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
         <is>
           <t>문선생 (322)
 M1-Elephantus</t>
@@ -1331,10 +1331,10 @@
     <row r="10">
       <c r="AC10" t="inlineStr">
         <is>
-          <t>5:00~5:55</t>
-        </is>
-      </c>
-      <c r="AG10" t="inlineStr">
+          <t>7:00~7:55</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
         <is>
           <t>양선생 (323)
 E4-Theseus</t>
@@ -1344,10 +1344,10 @@
     <row r="11">
       <c r="AC11" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="AH11" t="inlineStr">
+          <t>7:00~7:55</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
         <is>
           <t>양선생 (323)
 E5-Artemis</t>
@@ -1360,7 +1360,7 @@
           <t>7:00~7:55</t>
         </is>
       </c>
-      <c r="AD12" t="inlineStr">
+      <c r="AF12" t="inlineStr">
         <is>
           <t>양선생 (323)
 E6-Helios</t>
@@ -1370,10 +1370,10 @@
     <row r="13">
       <c r="AC13" t="inlineStr">
         <is>
-          <t>8:00~8:55</t>
-        </is>
-      </c>
-      <c r="AE13" t="inlineStr">
+          <t>7:00~7:55</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
         <is>
           <t>양선생 (323)
 M1-Elephantus</t>
@@ -1383,10 +1383,10 @@
     <row r="14">
       <c r="AC14" t="inlineStr">
         <is>
-          <t>3:00~3:55</t>
-        </is>
-      </c>
-      <c r="AF14" t="inlineStr">
+          <t>8:00~8:55</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
         <is>
           <t>배선생 (324)
 E4-Theseus</t>
@@ -1396,7 +1396,7 @@
     <row r="15">
       <c r="AC15" t="inlineStr">
         <is>
-          <t>4:00~4:55</t>
+          <t>8:00~8:55</t>
         </is>
       </c>
       <c r="AG15" t="inlineStr">
@@ -1409,10 +1409,10 @@
     <row r="16">
       <c r="AC16" t="inlineStr">
         <is>
-          <t>5:00~5:55</t>
-        </is>
-      </c>
-      <c r="AH16" t="inlineStr">
+          <t>8:00~8:55</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
         <is>
           <t>배선생 (324)
 E6-Helios</t>
@@ -1422,10 +1422,10 @@
     <row r="17">
       <c r="AC17" t="inlineStr">
         <is>
-          <t>6:00~6:55</t>
-        </is>
-      </c>
-      <c r="AD17" t="inlineStr">
+          <t>8:00~8:55</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
         <is>
           <t>배선생 (324)
 M1-Elephantus</t>

</xml_diff>